<commit_message>
Add test suite and CI workflow
- tests/test_convert.py: 56 pytest cases covering all 8 suffix rules
  (SingleList, ColorChoice, MultiList, Composite, Float, Boolean,
  Integer, MultiEntry) plus plain passthrough and parse_header
- .github/workflows/ci.yml: runs pytest on push/PR against Python 3.9, 3.11, 3.13
- Fix Integer validator to correctly accept negative whole numbers
- Update Load-Template.xlsx sample data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Load-Template.xlsx
+++ b/Load-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrem\Documents\Cowork\Code\plmdataloader\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D637DF7-EAB7-4801-B1B0-6D53FC942B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6562EEA5-D66B-4FB6-ACD8-BF527E42459E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{95216A6E-F2C4-4BA8-9D78-9FCC63A7CE89}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
   <si>
     <t>Object</t>
   </si>
@@ -178,6 +178,15 @@
   </si>
   <si>
     <t>Regions-MultiEntry</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>Class 4</t>
   </si>
 </sst>
 </file>
@@ -620,7 +629,7 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F2" t="s">
         <v>31</v>
@@ -669,8 +678,8 @@
       <c r="I3" t="s">
         <v>38</v>
       </c>
-      <c r="J3">
-        <v>500</v>
+      <c r="J3" t="s">
+        <v>47</v>
       </c>
       <c r="K3" t="s">
         <v>43</v>
@@ -698,8 +707,8 @@
       <c r="G4" t="s">
         <v>40</v>
       </c>
-      <c r="H4">
-        <v>4.5</v>
+      <c r="H4" t="s">
+        <v>46</v>
       </c>
       <c r="I4" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Doc: Updated sample excel file
</commit_message>
<xml_diff>
--- a/Load-Template.xlsx
+++ b/Load-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrem\Documents\Cowork\Code\plmdataloader\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6562EEA5-D66B-4FB6-ACD8-BF527E42459E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71ED610-3475-4450-9CE4-24036023C1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{95216A6E-F2C4-4BA8-9D78-9FCC63A7CE89}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t>Object</t>
   </si>
@@ -138,9 +138,6 @@
     <t>6 plus</t>
   </si>
   <si>
-    <t>Product</t>
-  </si>
-  <si>
     <t>Product\Type1</t>
   </si>
   <si>
@@ -180,13 +177,7 @@
     <t>Regions-MultiEntry</t>
   </si>
   <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>ok</t>
-  </si>
-  <si>
-    <t>Class 4</t>
+    <t>LCSProduct</t>
   </si>
 </sst>
 </file>
@@ -569,7 +560,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.08984375" customWidth="1"/>
     <col min="4" max="4" width="19.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.81640625" bestFit="1" customWidth="1"/>
@@ -609,56 +600,56 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
       </c>
       <c r="D2" t="s">
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
         <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H2">
         <v>3.05</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J2">
         <v>100</v>
       </c>
       <c r="K2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
         <v>32</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>34</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -667,33 +658,33 @@
         <v>25</v>
       </c>
       <c r="F3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
         <v>36</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
       </c>
       <c r="H3">
         <v>1.65</v>
       </c>
       <c r="I3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" t="s">
-        <v>47</v>
+        <v>37</v>
+      </c>
+      <c r="J3">
+        <v>400</v>
       </c>
       <c r="K3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>33</v>
-      </c>
-      <c r="C4" t="s">
-        <v>34</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
@@ -705,19 +696,19 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" t="s">
-        <v>46</v>
+        <v>39</v>
+      </c>
+      <c r="H4">
+        <v>4.5</v>
       </c>
       <c r="I4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J4">
         <v>600</v>
       </c>
       <c r="K4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -794,7 +785,7 @@
         <v>28</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Fix: Error handling mechanism
</commit_message>
<xml_diff>
--- a/Load-Template.xlsx
+++ b/Load-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrem\Documents\Cowork\Code\plmdataloader\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71ED610-3475-4450-9CE4-24036023C1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84097FED-B6A9-4046-AE32-72C8D0B5FDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{95216A6E-F2C4-4BA8-9D78-9FCC63A7CE89}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
   <si>
     <t>Object</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>LCSProduct</t>
+  </si>
+  <si>
+    <t>Class 4</t>
   </si>
 </sst>
 </file>
@@ -690,7 +693,7 @@
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Doc: updated validation rule for Composite
</commit_message>
<xml_diff>
--- a/Load-Template.xlsx
+++ b/Load-Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjrem\Documents\Cowork\Code\plmdataloader\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84097FED-B6A9-4046-AE32-72C8D0B5FDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1499BAE-5AF0-4B5F-9568-09C5E09466AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{95216A6E-F2C4-4BA8-9D78-9FCC63A7CE89}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{95216A6E-F2C4-4BA8-9D78-9FCC63A7CE89}"/>
   </bookViews>
   <sheets>
     <sheet name="Load Template" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
   <si>
     <t>Object</t>
   </si>
@@ -181,6 +181,42 @@
   </si>
   <si>
     <t>Class 4</t>
+  </si>
+  <si>
+    <t>Material Content-Composite</t>
+  </si>
+  <si>
+    <t>50% Cotton,50% Polyester</t>
+  </si>
+  <si>
+    <t>100% Polyester</t>
+  </si>
+  <si>
+    <t>100% Nylon</t>
+  </si>
+  <si>
+    <t>Material Content-Display Name</t>
+  </si>
+  <si>
+    <t>Material Content-Internal Name</t>
+  </si>
+  <si>
+    <t>xyzCotton</t>
+  </si>
+  <si>
+    <t>xyzPolyester</t>
+  </si>
+  <si>
+    <t>xyzNylon</t>
+  </si>
+  <si>
+    <t>Nylon</t>
+  </si>
+  <si>
+    <t>Polyester</t>
+  </si>
+  <si>
+    <t>Cotton</t>
   </si>
 </sst>
 </file>
@@ -559,7 +595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A38F08B4-D7DF-4B2C-8557-1E35A3BB5B94}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.36328125" bestFit="1" customWidth="1"/>
@@ -568,13 +604,14 @@
     <col min="5" max="5" width="13.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -597,19 +634,22 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -631,20 +671,23 @@
       <c r="G2" t="s">
         <v>36</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2">
         <v>3.05</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>38</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>100</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -666,20 +709,23 @@
       <c r="G3" t="s">
         <v>36</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3">
         <v>1.65</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>37</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>400</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -701,16 +747,19 @@
       <c r="G4" t="s">
         <v>39</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4">
         <v>4.5</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>37</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>600</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>43</v>
       </c>
     </row>
@@ -721,7 +770,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F89CC34-93AD-4022-9C3F-A4DC93190AD3}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
@@ -729,9 +778,10 @@
     <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -750,8 +800,14 @@
       <c r="F1" t="s">
         <v>14</v>
       </c>
+      <c r="G1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -770,8 +826,14 @@
       <c r="F2" t="s">
         <v>30</v>
       </c>
+      <c r="G2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -790,8 +852,14 @@
       <c r="F3" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="G3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" t="s">
+        <v>57</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -809,6 +877,12 @@
       </c>
       <c r="F4" t="s">
         <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>